<commit_message>
feat(m4): add keyword search and category filter with tests
</commit_message>
<xml_diff>
--- a/test-evidence/M4-Jia-Kaifan/UT-M4-table.xlsx
+++ b/test-evidence/M4-Jia-Kaifan/UT-M4-table.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="39">
   <si>
     <t>Test Name/ID</t>
   </si>
@@ -101,16 +101,46 @@
     <t>Sprint 2</t>
   </si>
   <si>
+    <t>An available topic exists with keyword "Java" under categoryId = 1</t>
+  </si>
+  <si>
+    <t>searchAvailableTopics("Java", 1L)</t>
+  </si>
+  <si>
+    <t>Returns matching available topics list</t>
+  </si>
+  <si>
+    <t>Method returns a list with 1 matching topic titled "Java Web Project"</t>
+  </si>
+  <si>
+    <t>Method returned a list with 1 topic, title = "Java Web Project"</t>
+  </si>
+  <si>
+    <t>UT-M4-S2-02</t>
+  </si>
+  <si>
+    <t>No available topic exists with keyword "Python" under categoryId = 2</t>
+  </si>
+  <si>
+    <t>searchAvailableTopics("Python", 2L)</t>
+  </si>
+  <si>
+    <t>Returns empty topics list</t>
+  </si>
+  <si>
+    <t>Method returns an empty list when no matching topic exists</t>
+  </si>
+  <si>
+    <t>Method returned an empty list</t>
+  </si>
+  <si>
+    <t>UT-M4-S3-01</t>
+  </si>
+  <si>
+    <t>Sprint 3</t>
+  </si>
+  <si>
     <t/>
-  </si>
-  <si>
-    <t>UT-M4-S2-02</t>
-  </si>
-  <si>
-    <t>UT-M4-S3-01</t>
-  </si>
-  <si>
-    <t>Sprint 3</t>
   </si>
   <si>
     <t>UT-M4-S3-02</t>
@@ -126,7 +156,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -138,13 +168,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -294,7 +317,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -322,12 +345,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -624,67 +641,70 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -699,77 +719,74 @@
     <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -781,6 +798,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1226,101 +1249,101 @@
       <c r="B4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>24</v>
+      <c r="D4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>24</v>
+      <c r="C5" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:8">
       <c r="A7" s="2" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>